<commit_message>
Update HORIZONS staff cleanup tracker workbooks
</commit_message>
<xml_diff>
--- a/HORIZONS_Missing_Info_Questions_Tracker.xlsx
+++ b/HORIZONS_Missing_Info_Questions_Tracker.xlsx
@@ -1,16 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions To Answer" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Missing Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions To Answer" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Staff Cleanup 2026-06-01" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Staff Cleanup 2026-06-01'!$A$1:$E$10</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +33,11 @@
       <b val="1"/>
       <color rgb="001F1F1F"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +47,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F3EAE1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,11 +67,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,7 +531,6 @@
           <t>Samuel / Aream &amp; Co.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>High</t>
@@ -530,7 +541,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Do not use the old name in live display unless confirmed as a separate person.</t>
@@ -563,7 +573,6 @@
           <t>Samuel / Chris / Venue</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>High</t>
@@ -574,7 +583,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Include phone, WhatsApp, venue contact, and escalation notes.</t>
@@ -607,7 +615,6 @@
           <t>Venue / Operations</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>High</t>
@@ -618,7 +625,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Use Google Maps Link Needed / Exact pin needed until supplied.</t>
@@ -651,7 +657,6 @@
           <t>Samuel / Venue</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -662,7 +667,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Weather location needs confirmation remains in notes.</t>
@@ -695,7 +699,6 @@
           <t>Creative / Guest Experience</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -706,7 +709,6 @@
           <t>File Needed</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Placeholder remains on site.</t>
@@ -739,7 +741,6 @@
           <t>Samuel / Guest Experience</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -750,7 +751,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Do not finalize naming until confirmed.</t>
@@ -783,7 +783,6 @@
           <t>Samuel / Guest Experience</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -794,7 +793,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Flagged on site.</t>
@@ -827,7 +825,6 @@
           <t>Samuel / Production</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>High</t>
@@ -838,7 +835,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Includes guest runner, prep owner, microphone and powder/makeup checks.</t>
@@ -871,7 +867,6 @@
           <t>Production</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>High</t>
@@ -882,7 +877,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>Confirm required people and owner.</t>
@@ -915,7 +909,6 @@
           <t>Creative / Clownfish</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>High</t>
@@ -926,7 +919,6 @@
           <t>File Needed</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>Site has placeholders for Map Needed / Location Needed / Placement Needed.</t>
@@ -959,7 +951,6 @@
           <t>Samuel / Chris</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>High</t>
@@ -970,7 +961,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>Production Slack routes remain disabled/test-mode until approved.</t>
@@ -1087,8 +1077,6 @@
           <t>Samuel / Venue</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -1099,8 +1087,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1128,8 +1114,6 @@
           <t>Samuel / Chris</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>High</t>
@@ -1140,8 +1124,6 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1169,8 +1151,6 @@
           <t>Guest Experience</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -1181,10 +1161,300 @@
           <t>Needs Confirmation</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="76" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Staff Lists</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Regroup staff into International Collective / I.N.C, Clownfish, Aream &amp; Co., B Good, Performers, Hotel / Venue</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Team-facing website data updated in content.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Clownfish</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Roles, dietary notes, and show-operative assignments</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HORIZONS Hall: George Winning + Ryan Lowe. HORIZONS Studio: Alex Hudson + Nathan Rushmer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>All team-facing views</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dates of birth excluded from website display and reports</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No date values are included in this tracker note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Nathan Rushmer email</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Email Needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>George Winning email</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Email Needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Joshua Millar email</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Email Needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ryan Lowe email and dietary final</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Email Needed; dietary TBC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Joachim Ridley-Barker email</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Email Needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alex Hudson email</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Email Needed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>